<commit_message>
update: student reports updated.
</commit_message>
<xml_diff>
--- a/student_report.xlsx
+++ b/student_report.xlsx
@@ -570,7 +570,7 @@
         <v>91</v>
       </c>
       <c r="G5" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="D6" t="n">
         <v>90</v>
@@ -597,10 +597,10 @@
         <v>93</v>
       </c>
       <c r="F6" t="n">
-        <v>91</v>
+        <v>92.5</v>
       </c>
       <c r="G6" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>

</xml_diff>